<commit_message>
V7-M1: compliance screens, draft deadline rules, acceptance package; DEC-089
* Screens: the client's Deadlines page (Compliance group in the workspace
  sidebar, behind practice.management) and the practice deadlines page with
  the API's counts; linked from the company list.
* Draft deadline rules (content/compliance/drafts, UNVERIFIED, not seeded)
  with scripts/compliance/import-deadline-rules.mjs; added to the verifier's
  worksheet ("Deadline rules" sheet).
* Tests: browser test tests/e2e/compliance.test.ts (5); API test of the pack
  import (lands UNVERIFIED, needs compliance:rules-manage).
* docs: v7-m1-acceptance.md (prepared; CI evidence follows),
  v7-compliance-matrix.md v1.0, DEC-089 (how V7-M2 is built, before code).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Cg1NTr1Jod9GiCK6MZqGU
</commit_message>
<xml_diff>
--- a/docs/legal/rule-verification-worksheet.xlsx
+++ b/docs/legal/rule-verification-worksheet.xlsx
@@ -10,8 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAT codes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standards and thresholds" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign-off" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legal references" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deadline rules" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign-off" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legal references" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -634,15 +635,37 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>Import content/compliance/drafts/uk-deadline-rules.json with scripts/compliance/import-deadline-rules.mjs, then check each rule on the 'Deadline rules' sheet and verify it, or supersede it with a corrected version first.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Import: a person with compliance:rules-manage; verify: Shoaib, with compliance:rule-verify</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>The platform refuses a verifier who entered the rule (DEC-088)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
           <t>Fill in the 'Sign-off' sheet with the platform's record of each verification.</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Shoaib</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Evidence for the go-live checklist (DEC-085, item 3)</t>
         </is>
@@ -1667,7 +1690,369 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Draft deadline rules (V7-M1, DEC-088)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Due date = anchor + days before, then + months (month-end rule: a month-end anchor stays a month end), then + days after. Import with scripts/compliance/import-deadline-rules.mjs; each lands UNVERIFIED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Legal forms</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Days before</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Months</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Days after</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Month-end rule</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Governs anchors from</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Provision to check</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>What the rule does not model</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Verified (yes / corrected)</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Verified on</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Verifier's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>ACCOUNTS_FILING</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>LTD, LLP</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Companies Act 2006 s.442(2)(a) (private company: 9 months after the end of the accounting reference period) and s.443 (month-end rule); applied to LLPs by SI 2008/1911. Drafted, not retrieved: check the period, the month-end treatment and the dates it governs against the text in force</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2006/46/section/442</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Private companies and LLPs only. A public company has 6 months (s.442(2)(b)) and is not modelled. First accounts (s.442(3), 21 months from incorporation) and shortened or extended periods are entered by hand with a reason (DEC-088).</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CT_PAYMENT</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>LTD</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Taxes Management Act 1970 s.59D (Corporation Tax due 9 months and 1 day after the end of the accounting period). Drafted, not retrieved: check the period, the month-end treatment and the dates it governs against the text in force</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/1970/9/section/59D</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Companies that are not large. Large and very large companies pay by quarterly instalments (SI 1998/3175), which are not modelled. LLPs do not pay Corporation Tax.</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr"/>
+      <c r="M6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>CT_RETURN</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>LTD</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Finance Act 1998 Sch 18 para 14 (Company Tax Return filing date: 12 months from the end of the period for which the return is made). Drafted, not retrieved: check the period, the month-end treatment and the dates it governs against the text in force</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/1998/36/schedule/18/paragraph/14</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Check whether para 14's later dates (3 months after the notice, long periods of account) need entering by hand. No month-end rule is assumed: check the treatment of 28 February.</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>CONFIRMATION_STATEMENT</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>LTD, LLP</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>2016-06-30</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Companies Act 2006 s.853A (confirmation statement delivered within 14 days after the end of the review period). Drafted, not retrieved: check the period, the month-end treatment and the dates it governs against the text in force</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2006/46/section/853A</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>The anchor is the confirmation date on the client's compliance profile (the end of the review period). Check the commencement date of the confirmation-statement regime.</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
+      <c r="M8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>VAT_RETURN</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>LTD, LLP, SOLE_TRADER, PARTNERSHIP, CHARITY, OTHER</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>2010-01-01</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>VAT Regulations 1995 reg 25(1) (return by the end of the month after the period) and HMRC's 7 extra days for electronic returns (Notice 700/12). Drafted, not retrieved: check the period, the month-end treatment and the dates it governs against the text in force</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/1995/2518/regulation/25</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Quarterly and monthly returns. The annual accounting scheme and payments on account are not modelled. Check that the 7-day extension applies to every client using the rule.</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId5"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1958,18 +2343,93 @@
       <c r="D20" s="6" t="inlineStr"/>
       <c r="E20" s="6" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>ACCOUNTS_FILING</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Deadline rule</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr"/>
+      <c r="D21" s="6" t="inlineStr"/>
+      <c r="E21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>CT_PAYMENT</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Deadline rule</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr"/>
+      <c r="D22" s="6" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>CT_RETURN</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Deadline rule</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr"/>
+      <c r="D23" s="6" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>CONFIRMATION_STATEMENT</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Deadline rule</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr"/>
+      <c r="D24" s="6" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>VAT_RETURN</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Deadline rule</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr"/>
+      <c r="D25" s="6" t="inlineStr"/>
+      <c r="E25" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -2113,66 +2573,100 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Small Companies and Groups (Accounts and Directors' Report) Regulations 2008, SI 2008/409</t>
+          <t>Companies Act 2006, ss.442-443 and 853A</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Formats and notes for small and micro-entity accounts</t>
+          <t>Deadlines: filing accounts, the month-end rule, the confirmation statement</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>https://www.legislation.gov.uk/uksi/2008/409/contents</t>
+          <t>https://www.legislation.gov.uk/ukpga/2006/46/section/442</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>FRS 105 and FRS 102 Section 1A (Financial Reporting Council)</t>
+          <t>Taxes Management Act 1970, s.59D; Finance Act 1998, Sch 18 para 14</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>The standards the draft packs follow</t>
+          <t>Deadlines: Corporation Tax payment and the Company Tax Return</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>https://www.frc.org.uk/accountants/accounting-and-reporting-policy/uk-accounting-standards</t>
+          <t>https://www.legislation.gov.uk/ukpga/1970/9/section/59D</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Card Protection Plan Ltd v Customs and Excise Commissioners (C-349/96)</t>
+          <t>Small Companies and Groups (Accounts and Directors' Report) Regulations 2008, SI 2008/409</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Single or multiple supplies: decides which code a sale takes</t>
+          <t>Formats and notes for small and micro-entity accounts</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:61996CJ0349</t>
+          <t>https://www.legislation.gov.uk/uksi/2008/409/contents</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>FRS 105 and FRS 102 Section 1A (Financial Reporting Council)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>The standards the draft packs follow</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.frc.org.uk/accountants/accounting-and-reporting-policy/uk-accounting-standards</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Card Protection Plan Ltd v Customs and Excise Commissioners (C-349/96)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Single or multiple supplies: decides which code a sale takes</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:61996CJ0349</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>Fiscale eenheid Koninklijke Ahold BV v Staatssecretaris van Financien (C-484/06)</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Rounding of VAT is a matter for national rules</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:62006CJ0484</t>
         </is>
@@ -2190,6 +2684,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V4-M1: Corporation Tax rules, tax periods and the tax profile (DEC-097, DEC-098)
- ct_rule (sourced, effective-dated, verified by a second person, immutable,
  superseded once, no overlap of current versions), company_tax_profile and
  ct_period (dates fixed, associated companies versioned); RLS, grants,
  retention
- CorporationTaxService and 11 API routes behind corporation.tax, in the
  OpenAPI contract; permissions ct:manage and ct:prepare
- Draft rule pack (UNVERIFIED) with its import tool and a worksheet sheet
- Unit, API and database tests; registries; acceptance package

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Cg1NTr1Jod9GiCK6MZqGU
</commit_message>
<xml_diff>
--- a/docs/legal/rule-verification-worksheet.xlsx
+++ b/docs/legal/rule-verification-worksheet.xlsx
@@ -13,8 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deadline rules" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAT presentation" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="iXBRL mapping" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign-off" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legal references" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corporation Tax rules" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign-off" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legal references" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -703,15 +704,37 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>Import content/tax/drafts/uk-ct-rules.json with scripts/tax/import-ct-rules.mjs, then check each rule on the 'Corporation Tax rules' sheet against its provision and verify it, or supersede it with a corrected version first.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Import: a person with ct:manage; verify: Shoaib, with tax:rule-verify</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>The platform refuses a verifier who entered the rule; CT periods cannot be derived until the period rule is verified (DEC-097)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
           <t>Fill in the 'Sign-off' sheet with the platform's record of each verification.</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Shoaib</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Evidence for the go-live checklist (DEC-085, item 3)</t>
         </is>
@@ -3808,7 +3831,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Draft Corporation Tax rules (V4-M1, DEC-097)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Import with scripts/tax/import-ct-rules.mjs; each lands UNVERIFIED. Rates are percentages, limits are pounds for a 12-month period with no associated companies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Effective from</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Effective to</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Parameters</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Provision to check</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>What to check</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Verified (yes / corrected)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Verified on</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Verifier's notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>CT_RATES</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2023-04-01</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>mainRate = 25; smallProfitsRate = 19; lowerLimit = 50000; upperLimit = 250000; marginalReliefFraction = 3/200</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>CTA 2010 Part 3A ss 18A-18N (small profits rate, limits, marginal relief), inserted by FA 2021 s 7 and Sch 1; main rate FA 2021 s 6</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2010/4/part/3A</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Check the main rate (25%) and the small profits rate (19%) against the charge for each financial year from FY2023 (FA 2021 s 6 for FY2023; the later Finance Acts charge each later year). Check the lower and upper limits (£50,000 and £250,000, for a 12-month period with no associated companies) and the standard marginal relief fraction 3/200. If a later year changes any figure, end this version on 31 March of the last year it covers and enter the new one. HMRC summary: https://www.gov.uk/government/publications/rates-and-allowances-corporation-tax</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>PERIOD_MAX_MONTHS</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>2009-04-01</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>months = 12</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>CTA 2009 s 10(1)(a): an accounting period ends on the expiry of 12 months from its beginning</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2009/4/section/10</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Check that a CT accounting period ends no later than 12 months from its start (CTA 2009 s 10(1)(a)). The platform splits a longer accounts year into a first period of 12 months from the year's start and a second period for the rest (HMRC Company Taxation Manual CTM01405).</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4204,18 +4395,48 @@
       <c r="D27" s="6" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>CT_RATES</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Corporation Tax rule</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr"/>
+      <c r="D28" s="6" t="inlineStr"/>
+      <c r="E28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>PERIOD_MAX_MONTHS</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Corporation Tax rule</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr"/>
+      <c r="D29" s="6" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -4444,83 +4665,168 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Taxes Management Act 1970, s.59D; Finance Act 1998, Sch 18 para 14</t>
+          <t>Corporation Tax Act 2009, s.10</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Deadlines: Corporation Tax payment and the Company Tax Return</t>
+          <t>When a CT accounting period ends: 12 months from its start at the latest</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>https://www.legislation.gov.uk/ukpga/1970/9/section/59D</t>
+          <t>https://www.legislation.gov.uk/ukpga/2009/4/section/10</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Small Companies and Groups (Accounts and Directors' Report) Regulations 2008, SI 2008/409</t>
+          <t>Corporation Tax Act 2010, Part 3A (ss.18A-18N), inserted by Finance Act 2021 s.7 and Sch 1</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Formats and notes for small and micro-entity accounts</t>
+          <t>The small profits rate, the lower and upper limits, associated companies and marginal relief</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>https://www.legislation.gov.uk/uksi/2008/409/contents</t>
+          <t>https://www.legislation.gov.uk/ukpga/2010/4/part/3A</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>FRS 105 and FRS 102 Section 1A (Financial Reporting Council)</t>
+          <t>Finance Act 2021, s.6</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>The standards the draft packs follow</t>
+          <t>The main rate of 25% for the financial year 2023</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>https://www.frc.org.uk/accountants/accounting-and-reporting-policy/uk-accounting-standards</t>
+          <t>https://www.legislation.gov.uk/ukpga/2021/26/section/6</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Card Protection Plan Ltd v Customs and Excise Commissioners (C-349/96)</t>
+          <t>HMRC: Rates and allowances for Corporation Tax</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Single or multiple supplies: decides which code a sale takes</t>
+          <t>HMRC's summary of the rates and limits by financial year</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:61996CJ0349</t>
+          <t>https://www.gov.uk/government/publications/rates-and-allowances-corporation-tax</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>HMRC Company Taxation Manual CTM01405</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Accounting periods: a period of account longer than 12 months</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/hmrc-internal-manuals/company-taxation-manual/ctm01405</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Taxes Management Act 1970, s.59D; Finance Act 1998, Sch 18 para 14</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Deadlines: Corporation Tax payment and the Company Tax Return</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/1970/9/section/59D</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Small Companies and Groups (Accounts and Directors' Report) Regulations 2008, SI 2008/409</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Formats and notes for small and micro-entity accounts</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2008/409/contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>FRS 105 and FRS 102 Section 1A (Financial Reporting Council)</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>The standards the draft packs follow</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>https://www.frc.org.uk/accountants/accounting-and-reporting-policy/uk-accounting-standards</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Card Protection Plan Ltd v Customs and Excise Commissioners (C-349/96)</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Single or multiple supplies: decides which code a sale takes</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:61996CJ0349</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
           <t>Fiscale eenheid Koninklijke Ahold BV v Staatssecretaris van Financien (C-484/06)</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Rounding of VAT is a matter for national rules</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:62006CJ0484</t>
         </is>
@@ -4544,6 +4850,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V4-M3: capital allowances (DEC-100); CI evidence for V3 and V4-M1
- CT rule kinds AIA_LIMIT, WDA_RATES and SMALL_POOL_LIMIT (draft pack
  extended, UNVERIFIED); computeCapitalAllowances in pennies: AIA in date
  order, main and special rate pools, single asset pools, disposal values
  capped at cost, small pools, balancing allowances and charges, the
  fraction of a short period
- ca_pool_opening (evidence, second-person verification, immutable) and
  ca_computation (stored as read, chained to the prior period, superseded
  once, stale marks); RLS, grants, retention
- 7 API routes behind corporation.tax, in the OpenAPI contract
- A two-period golden (JSON and formula workbook), unit and API tests,
  registries, acceptance package
- Run 203 recorded: V3-M1, V3-M3, V3-M4 and V4-M1 accepted; V3-M2 green,
  awaiting the accountant's review of its golden tagging

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Cg1NTr1Jod9GiCK6MZqGU
</commit_message>
<xml_diff>
--- a/docs/legal/rule-verification-worksheet.xlsx
+++ b/docs/legal/rule-verification-worksheet.xlsx
@@ -3831,7 +3831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3984,10 +3984,121 @@
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>AIA_LIMIT</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>2023-04-01</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>annualLimit = 1000000</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>CAA 2001 s 51A(5): the maximum allowance of £1,000,000, made permanent from 1 April 2023</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2001/2/section/51A</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Check the £1,000,000 annual investment allowance limit and the date it applies from, and the Finance Act that made it permanent. The platform scales it by days/365 for a period shorter than 12 months (CAA 2001 s 51E); a period spanning a change of limit is refused, not apportioned (s 51B-51D style transitional rules are not modelled).</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>WDA_RATES</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2019-04-01</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>mainRate = 18; specialRate = 6</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>CAA 2001 s 56(1) (main pool 18%) and s 104D (special rate pool 6% from April 2019)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2001/2/section/56</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Check the main pool rate (18%) and the special rate (6%, reduced from 8% for chargeable periods from 1 April 2019; s 104D). The platform scales the allowance by days/365 for a period shorter than 12 months (s 56(3)); hybrid rates for a period spanning a change are not modelled.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>SMALL_POOL_LIMIT</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2008-04-01</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>limit = 1000</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>CAA 2001 s 56A: small pools allowance where unrelieved expenditure is £1,000 or less</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/2001/2/section/56A</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Check the £1,000 small pools limit (main and special rate pools only) and its reduction for a period shorter than 12 months. The platform claims it whenever it applies; a claim is optional in law and disclaiming is not modelled.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3999,7 +4110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4425,6 +4536,51 @@
       <c r="D29" s="6" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr"/>
     </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>AIA_LIMIT</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Corporation Tax rule</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr"/>
+      <c r="D30" s="6" t="inlineStr"/>
+      <c r="E30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>WDA_RATES</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Corporation Tax rule</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr"/>
+      <c r="D31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>SMALL_POOL_LIMIT</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Corporation Tax rule</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr"/>
+      <c r="D32" s="6" t="inlineStr"/>
+      <c r="E32" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4436,7 +4592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -4750,83 +4906,151 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Taxes Management Act 1970, s.59D; Finance Act 1998, Sch 18 para 14</t>
+          <t>Capital Allowances Act 2001, ss.51A-51E (annual investment allowance)</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Deadlines: Corporation Tax payment and the Company Tax Return</t>
+          <t>The AIA limit and its reduction for a short period</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>https://www.legislation.gov.uk/ukpga/1970/9/section/59D</t>
+          <t>https://www.legislation.gov.uk/ukpga/2001/2/section/51A</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Small Companies and Groups (Accounts and Directors' Report) Regulations 2008, SI 2008/409</t>
+          <t>Capital Allowances Act 2001, ss.56, 56A and 104D</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Formats and notes for small and micro-entity accounts</t>
+          <t>Writing-down allowances (main 18%, special rate 6%), the small pools allowance</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>https://www.legislation.gov.uk/uksi/2008/409/contents</t>
+          <t>https://www.legislation.gov.uk/ukpga/2001/2/section/56</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>FRS 105 and FRS 102 Section 1A (Financial Reporting Council)</t>
+          <t>Capital Allowances Act 2001, ss.61-62</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>The standards the draft packs follow</t>
+          <t>Disposal values, capped at the qualifying expenditure</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>https://www.frc.org.uk/accountants/accounting-and-reporting-policy/uk-accounting-standards</t>
+          <t>https://www.legislation.gov.uk/ukpga/2001/2/section/62</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Card Protection Plan Ltd v Customs and Excise Commissioners (C-349/96)</t>
+          <t>HMRC Capital Allowances Manual CA23000 onwards (plant and machinery)</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Single or multiple supplies: decides which code a sale takes</t>
+          <t>HMRC's guidance on pools, AIA and writing-down allowances</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:61996CJ0349</t>
+          <t>https://www.gov.uk/hmrc-internal-manuals/capital-allowances-manual/ca23000</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
+          <t>Taxes Management Act 1970, s.59D; Finance Act 1998, Sch 18 para 14</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Deadlines: Corporation Tax payment and the Company Tax Return</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/ukpga/1970/9/section/59D</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Small Companies and Groups (Accounts and Directors' Report) Regulations 2008, SI 2008/409</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Formats and notes for small and micro-entity accounts</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>https://www.legislation.gov.uk/uksi/2008/409/contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>FRS 105 and FRS 102 Section 1A (Financial Reporting Council)</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>The standards the draft packs follow</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>https://www.frc.org.uk/accountants/accounting-and-reporting-policy/uk-accounting-standards</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Card Protection Plan Ltd v Customs and Excise Commissioners (C-349/96)</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Single or multiple supplies: decides which code a sale takes</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:61996CJ0349</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
           <t>Fiscale eenheid Koninklijke Ahold BV v Staatssecretaris van Financien (C-484/06)</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Rounding of VAT is a matter for national rules</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:62006CJ0484</t>
         </is>
@@ -4855,6 +5079,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
V4-M5: CT iXBRL and the HMRC submission through a fake adapter (DEC-102)
- CT600_FORM rule kind (the box of each canonical field, verified) with a
  draft map in the pack (UNVERIFIED); two totals added to the canonical
  CT600 (tax at the rates, marginal relief)
- buildCtIxbrl: the computation as inline XBRL from a verified CT-COMP
  taxonomy version; contexts for the period and each financial-year part;
  the UTR as the entity identifier
- ct_return (package frozen at creation, path guarded in the database,
  second-person director's declaration) and ct_return_event (append-only);
  the HMRC CT port with a fake adapter only (HMRC_CT_ADAPTER, refused in
  production); acceptance closes the CT_RETURN obligation
- Permission ct:file; 9 API routes behind corporation.tax, in the OpenAPI
  contract; unit and API tests (xmllint), registries, acceptance package

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015Cg1NTr1Jod9GiCK6MZqGU
</commit_message>
<xml_diff>
--- a/docs/legal/rule-verification-worksheet.xlsx
+++ b/docs/legal/rule-verification-worksheet.xlsx
@@ -3831,7 +3831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4092,6 +4092,42 @@
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>CT600_FORM</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2015-04-01</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>CT600 (2015) version 3 (draft map): turnover -&gt; box 145, tradingProfits -&gt; box 155, tradingLossesBroughtForwardUsed -&gt; box 160, netTradingProfits -&gt; box 165, nonTradingLoanRelationships -&gt; box 170, propertyIncome -&gt; box 190, chargeableGains -&gt; box 210, taxableTotalProfits -&gt; box 315, associatedCompanies -&gt; box 326, fy1.financialYear -&gt; box 330, fy1.profit -&gt; box 335, fy1.rate -&gt; box 340, fy1.taxAtRate -&gt; box 345, fy2.financialYear -&gt; box 380, fy2.profit -&gt; box 385, fy2.rate -&gt; box 390, fy2.taxAtRate -&gt; box 395, corporationTaxAtRates -&gt; box 430, marginalReliefTotal -&gt; box 435, corporationTaxChargeable -&gt; box 440, taxPayable -&gt; box 525</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>HMRC form CT600 (2015) version 3 and its guide (CT600 Guide)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/corporation-tax-company-tax-return-ct600-2015-version-3</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Engineering's draft box map, written from memory and not checked against the form. Check every box against the current CT600 and its guide, including the version in use for the period. Fields with no box here (the loss carried back from a later period, the trading loss of the period, losses carried back and forward, and the marginal relief and associated-company boxes per financial year) make a return with a value in them refuse to start until you map them: losses are on the supplementary pages and the loss boxes of the form. Correct the map by superseding it before verifying.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
@@ -4099,6 +4135,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4110,7 +4147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4581,6 +4618,21 @@
       <c r="D32" s="6" t="inlineStr"/>
       <c r="E32" s="6" t="inlineStr"/>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>CT600_FORM</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Corporation Tax rule</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr"/>
+      <c r="D33" s="6" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4592,7 +4644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -4974,83 +5026,100 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Taxes Management Act 1970, s.59D; Finance Act 1998, Sch 18 para 14</t>
+          <t>HMRC form CT600 (2015) version 3 and the CT600 Guide</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Deadlines: Corporation Tax payment and the Company Tax Return</t>
+          <t>The boxes of the Company Tax Return that the CT600_FORM rule maps</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>https://www.legislation.gov.uk/ukpga/1970/9/section/59D</t>
+          <t>https://www.gov.uk/government/publications/corporation-tax-company-tax-return-ct600-2015-version-3</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Small Companies and Groups (Accounts and Directors' Report) Regulations 2008, SI 2008/409</t>
+          <t>Taxes Management Act 1970, s.59D; Finance Act 1998, Sch 18 para 14</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Formats and notes for small and micro-entity accounts</t>
+          <t>Deadlines: Corporation Tax payment and the Company Tax Return</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>https://www.legislation.gov.uk/uksi/2008/409/contents</t>
+          <t>https://www.legislation.gov.uk/ukpga/1970/9/section/59D</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>FRS 105 and FRS 102 Section 1A (Financial Reporting Council)</t>
+          <t>Small Companies and Groups (Accounts and Directors' Report) Regulations 2008, SI 2008/409</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>The standards the draft packs follow</t>
+          <t>Formats and notes for small and micro-entity accounts</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>https://www.frc.org.uk/accountants/accounting-and-reporting-policy/uk-accounting-standards</t>
+          <t>https://www.legislation.gov.uk/uksi/2008/409/contents</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Card Protection Plan Ltd v Customs and Excise Commissioners (C-349/96)</t>
+          <t>FRS 105 and FRS 102 Section 1A (Financial Reporting Council)</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Single or multiple supplies: decides which code a sale takes</t>
+          <t>The standards the draft packs follow</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:61996CJ0349</t>
+          <t>https://www.frc.org.uk/accountants/accounting-and-reporting-policy/uk-accounting-standards</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
+          <t>Card Protection Plan Ltd v Customs and Excise Commissioners (C-349/96)</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Single or multiple supplies: decides which code a sale takes</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:61996CJ0349</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
           <t>Fiscale eenheid Koninklijke Ahold BV v Staatssecretaris van Financien (C-484/06)</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Rounding of VAT is a matter for national rules</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>https://eur-lex.europa.eu/legal-content/EN/TXT/?uri=CELEX:62006CJ0484</t>
         </is>
@@ -5083,6 +5152,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>